<commit_message>
updated chunking based on new data
</commit_message>
<xml_diff>
--- a/chunking/chunking_evaluation.xlsx
+++ b/chunking/chunking_evaluation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TongQuan_SoSanh" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ChiTiet_TungVanBan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PhanBo_KichThuoc" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DeXuat_QuyTac" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TongQuan_SoSanh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChiTiet_TungVanBan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhanBo_KichThuoc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeXuat_QuyTac" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,32 +507,32 @@
         <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>588</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>1470</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H2" t="n">
-        <v>220.7</v>
+        <v>796.5</v>
       </c>
       <c r="I2" t="n">
-        <v>349</v>
+        <v>3265</v>
       </c>
       <c r="J2" t="n">
-        <v>22.5</v>
+        <v>67.5</v>
       </c>
       <c r="K2" t="n">
-        <v>31</v>
+        <v>246</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -557,32 +557,32 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>925</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>1794</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1.94</v>
       </c>
       <c r="H3" t="n">
-        <v>220.7</v>
+        <v>541.8</v>
       </c>
       <c r="I3" t="n">
-        <v>349</v>
+        <v>2608</v>
       </c>
       <c r="J3" t="n">
-        <v>22.5</v>
+        <v>56.7</v>
       </c>
       <c r="K3" t="n">
-        <v>31</v>
+        <v>114</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>663</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>86.8%</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -607,32 +607,32 @@
         <v>30</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>501</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>1304</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2.6</v>
       </c>
       <c r="H4" t="n">
-        <v>220.7</v>
+        <v>916.2</v>
       </c>
       <c r="I4" t="n">
-        <v>349</v>
+        <v>2583</v>
       </c>
       <c r="J4" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="K4" t="n">
-        <v>44</v>
+        <v>381</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>67.1%</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -657,32 +657,32 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>588</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>1550</v>
       </c>
       <c r="G5" t="n">
-        <v>2.33</v>
+        <v>2.64</v>
       </c>
       <c r="H5" t="n">
-        <v>220.7</v>
+        <v>796.5</v>
       </c>
       <c r="I5" t="n">
-        <v>349</v>
+        <v>3265</v>
       </c>
       <c r="J5" t="n">
-        <v>19.3</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>74.1%</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -775,86 +775,559 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sample_documents_0</t>
+          <t>validated_L02</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>230</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2.05</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>138</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>252</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>1.83</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>111</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>216</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1.95</v>
       </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>249</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>validated_ND04</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>53</v>
+      </c>
+      <c r="C3" t="n">
+        <v>154</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="E3" t="n">
+        <v>105</v>
+      </c>
+      <c r="F3" t="n">
+        <v>187</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H3" t="n">
+        <v>39</v>
+      </c>
+      <c r="I3" t="n">
+        <v>127</v>
+      </c>
+      <c r="J3" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="K3" t="n">
+        <v>53</v>
+      </c>
+      <c r="L3" t="n">
+        <v>163</v>
+      </c>
+      <c r="M3" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>validated_ND05</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>38</v>
+      </c>
+      <c r="C4" t="n">
+        <v>97</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="E4" t="n">
+        <v>59</v>
+      </c>
+      <c r="F4" t="n">
+        <v>112</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I4" t="n">
+        <v>96</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="K4" t="n">
+        <v>38</v>
+      </c>
+      <c r="L4" t="n">
+        <v>101</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2.66</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>luat_52_2014_qh13</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>137</v>
+      </c>
+      <c r="C5" t="n">
+        <v>373</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E5" t="n">
+        <v>192</v>
+      </c>
+      <c r="F5" t="n">
+        <v>397</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="H5" t="n">
+        <v>133</v>
+      </c>
+      <c r="I5" t="n">
+        <v>338</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="K5" t="n">
+        <v>137</v>
+      </c>
+      <c r="L5" t="n">
+        <v>397</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nd_126_2014_nd_cp</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C6" t="n">
+        <v>254</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="E6" t="n">
+        <v>150</v>
+      </c>
+      <c r="F6" t="n">
+        <v>297</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="H6" t="n">
+        <v>73</v>
+      </c>
+      <c r="I6" t="n">
+        <v>229</v>
+      </c>
+      <c r="J6" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="K6" t="n">
+        <v>87</v>
+      </c>
+      <c r="L6" t="n">
+        <v>261</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>nd_158_2005_nd_cp</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>103</v>
+      </c>
+      <c r="F7" t="n">
+        <v>142</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="H7" t="n">
+        <v>31</v>
+      </c>
+      <c r="I7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="K7" t="n">
+        <v>50</v>
+      </c>
+      <c r="L7" t="n">
+        <v>96</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.92</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nd_207_2025_nd_cp</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>31</v>
+      </c>
+      <c r="C8" t="n">
+        <v>81</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="E8" t="n">
+        <v>60</v>
+      </c>
+      <c r="F8" t="n">
+        <v>99</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="H8" t="n">
+        <v>24</v>
+      </c>
+      <c r="I8" t="n">
+        <v>70</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="K8" t="n">
+        <v>31</v>
+      </c>
+      <c r="L8" t="n">
+        <v>85</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2.74</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>nq_01_2024_nq_hdtp</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" t="n">
+        <v>68</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>32</v>
+      </c>
+      <c r="F9" t="n">
+        <v>114</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="H9" t="n">
+        <v>17</v>
+      </c>
+      <c r="I9" t="n">
+        <v>54</v>
+      </c>
+      <c r="J9" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="K9" t="n">
+        <v>25</v>
+      </c>
+      <c r="L9" t="n">
+        <v>68</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tt_32_2016_tt_byt</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>6</v>
+      </c>
+      <c r="I10" t="n">
+        <v>17</v>
+      </c>
+      <c r="J10" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="K10" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" t="n">
+        <v>25</v>
+      </c>
+      <c r="M10" t="n">
+        <v>3.12</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tt_34_2017_tt_byt</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>12</v>
+      </c>
+      <c r="C11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="E11" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" t="n">
+        <v>9</v>
+      </c>
+      <c r="I11" t="n">
+        <v>33</v>
+      </c>
+      <c r="J11" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="K11" t="n">
+        <v>12</v>
+      </c>
+      <c r="L11" t="n">
+        <v>35</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2.92</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ttlt_01_2016_ttlt_tandtc</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>32</v>
+      </c>
+      <c r="C12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="E12" t="n">
+        <v>53</v>
+      </c>
+      <c r="F12" t="n">
+        <v>127</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>22</v>
+      </c>
+      <c r="I12" t="n">
+        <v>44</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32</v>
+      </c>
+      <c r="L12" t="n">
+        <v>62</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sample_documents_0</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>parsed_output_test</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C14" t="n">
         <v>5</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D14" t="n">
         <v>2.5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E14" t="n">
         <v>2</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F14" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G14" t="n">
         <v>2.5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H14" t="n">
         <v>2</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I14" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J14" t="n">
         <v>1.5</v>
       </c>
-      <c r="K3" t="n">
+      <c r="K14" t="n">
         <v>2</v>
       </c>
-      <c r="L3" t="n">
+      <c r="L14" t="n">
         <v>6</v>
       </c>
-      <c r="M3" t="n">
+      <c r="M14" t="n">
         <v>3</v>
       </c>
     </row>
@@ -931,30 +1404,30 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>1470</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>647</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>44.0%</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>709</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>48.2%</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>7.8%</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -973,22 +1446,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6</v>
+        <v>1794</v>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>838</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>46.7%</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>956</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>53.3%</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -1015,38 +1488,38 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>1304</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>496</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>38.0%</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>705</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>54.1%</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>2.8%</t>
         </is>
       </c>
     </row>
@@ -1057,30 +1530,30 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>1550</v>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>732</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>47.2%</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>704</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>45.4%</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>7.4%</t>
         </is>
       </c>
       <c r="I5" t="n">

</xml_diff>

<commit_message>
fix(chunking): stop using intro sentence as title for untitled articles
</commit_message>
<xml_diff>
--- a/chunking/chunking_evaluation.xlsx
+++ b/chunking/chunking_evaluation.xlsx
@@ -533,7 +533,7 @@
         <v>2.17</v>
       </c>
       <c r="I2" t="n">
-        <v>743.4</v>
+        <v>742.4</v>
       </c>
       <c r="J2" t="n">
         <v>1497</v>
@@ -577,7 +577,7 @@
         <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="G3" t="n">
         <v>2647</v>
@@ -586,7 +586,7 @@
         <v>1.96</v>
       </c>
       <c r="I3" t="n">
-        <v>529</v>
+        <v>528.6</v>
       </c>
       <c r="J3" t="n">
         <v>799</v>
@@ -639,7 +639,7 @@
         <v>2.36</v>
       </c>
       <c r="I4" t="n">
-        <v>842.5</v>
+        <v>841.3</v>
       </c>
       <c r="J4" t="n">
         <v>2497</v>
@@ -692,7 +692,7 @@
         <v>2.17</v>
       </c>
       <c r="I5" t="n">
-        <v>743.4</v>
+        <v>742.4</v>
       </c>
       <c r="J5" t="n">
         <v>1497</v>

</xml_diff>